<commit_message>
Insertar evidencias visuales en resultados manuales
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reportes/ejecucion-manual/Plantilla - Casos de prueba - ejecutada.xlsx
+++ b/reportes/ejecucion-manual/Plantilla - Casos de prueba - ejecutada.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24c0bad5dbd80ad4/Desktop/Proyecto-Aseguramiento y Calidad de software/048-proyecto-final/reportes/ejecucion-manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{4EF7628D-2600-4160-9ACF-98E5AD117BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77078EE2-7D1C-489D-BB1D-A7DD58097FDA}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{4EF7628D-2600-4160-9ACF-98E5AD117BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DBCA349-3370-498A-9647-9D765A34E176}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Suite de pruebas" sheetId="3" r:id="rId1"/>
+    <sheet name="Detalle de resultados" sheetId="4" r:id="rId1"/>
+    <sheet name="Suite de pruebas" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="101">
   <si>
     <t>OK</t>
   </si>
@@ -279,6 +280,75 @@
   </si>
   <si>
     <t>iPhone se agregó (1 unidad, $123.20) y retiró; carrito final vacío ($0.00). Al agregarlo apareció *** y un aviso de no disponibilidad aunque la ficha decía In Stock; reproducido 2 veces. Defecto confirmado BUG-002. Evidencia: CP-MAN-10-agregado.png, CP-MAN-10-repeticion.png y CP-MAN-10.png.</t>
+  </si>
+  <si>
+    <t>Caso</t>
+  </si>
+  <si>
+    <t>Resultado observado</t>
+  </si>
+  <si>
+    <t>Evidencia</t>
+  </si>
+  <si>
+    <t>CP-MAN-01</t>
+  </si>
+  <si>
+    <t>CP-MAN-01.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-02</t>
+  </si>
+  <si>
+    <t>CP-MAN-02.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-03</t>
+  </si>
+  <si>
+    <t>CP-MAN-03.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-04</t>
+  </si>
+  <si>
+    <t>CP-MAN-04.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-05</t>
+  </si>
+  <si>
+    <t>CP-MAN-05.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-06</t>
+  </si>
+  <si>
+    <t>CP-MAN-06.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-07</t>
+  </si>
+  <si>
+    <t>CP-MAN-07.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-08</t>
+  </si>
+  <si>
+    <t>CP-MAN-08.png; CP-MAN-08-repeticion.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-09</t>
+  </si>
+  <si>
+    <t>CP-MAN-09.png</t>
+  </si>
+  <si>
+    <t>CP-MAN-10</t>
+  </si>
+  <si>
+    <t>CP-MAN-10-agregado.png; CP-MAN-10-repeticion.png; CP-MAN-10.png</t>
   </si>
 </sst>
 </file>
@@ -317,7 +387,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -348,6 +418,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -361,7 +437,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -381,17 +457,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -405,6 +472,21 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -603,6 +685,511 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>67018</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>2158769</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Imagen 2" descr="CP-MAN-01 - CP-MAN-01.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{203D424C-C791-47FF-83D0-0468B0EEA3DC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="840741"/>
+          <a:ext cx="1846580" cy="2091751"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>68775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>2439710</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen 4" descr="CP-MAN-02 - CP-MAN-02.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A74E1F4-FDE9-418D-8D28-DFBC671DD4CB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="3058160"/>
+          <a:ext cx="1846580" cy="2370935"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>71121</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>2066504</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Imagen 6" descr="CP-MAN-03 - CP-MAN-03.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B359A4D4-75B4-447C-B1B8-24D98C6BF910}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="5557521"/>
+          <a:ext cx="1846580" cy="1995383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>76983</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>2072366</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Imagen 8" descr="CP-MAN-04 - CP-MAN-04.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1007AB3-49A5-483E-9512-97A6A9A6861B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="8605521"/>
+          <a:ext cx="1846580" cy="1995383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>76982</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>2172985</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Imagen 10" descr="CP-MAN-05 - CP-MAN-05.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FBCEE95-B9F5-4372-91C2-40EAF56A16F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="10739120"/>
+          <a:ext cx="1846580" cy="2096003"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>76396</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>2071779</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Imagen 12" descr="CP-MAN-06 - CP-MAN-06.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{956A9760-9636-44AB-A025-66703CA343B6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="12971781"/>
+          <a:ext cx="1846580" cy="1995383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>79912</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>2448013</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Imagen 14" descr="CP-MAN-07 - CP-MAN-07.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{222F6B78-988B-4EE5-9793-1A1001412D58}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="15654020"/>
+          <a:ext cx="1846580" cy="2368101"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>82258</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>2077641</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Imagen 16" descr="CP-MAN-08 - CP-MAN-08.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3DB37B0E-61B1-4EB1-A404-F037CEC5560B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="18153381"/>
+          <a:ext cx="1846580" cy="1995383"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>82257</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>2268959</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="19" name="Imagen 18" descr="CP-MAN-09 - CP-MAN-09.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B3F8BFD3-5C5E-4AE9-93A7-154B116895A6}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="20286980"/>
+          <a:ext cx="1846580" cy="2186702"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>61742</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>79326</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1908322</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>2294372</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="21" name="Imagen 20" descr="CP-MAN-10 - CP-MAN-10-repeticion.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79C2BECA-297E-4C4F-8F94-E0A0B3ACB6C7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="22611080"/>
+          <a:ext cx="1846580" cy="2215046"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -867,6 +1454,177 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F9ADDF-D33F-4C42-B5A1-5813E3A0ACA6}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
+    <col min="2" max="2" width="38.77734375" customWidth="1"/>
+    <col min="3" max="3" width="100.77734375" customWidth="1"/>
+    <col min="4" max="4" width="48.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -878,23 +1636,23 @@
     <col min="5" max="5" width="15.6640625" style="1" customWidth="1"/>
     <col min="6" max="6" width="27.33203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="36.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="38.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="28.77734375" style="1" customWidth="1"/>
     <col min="9" max="9" width="10.6640625" style="1" customWidth="1"/>
     <col min="10" max="16384" width="10.6640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
@@ -932,102 +1690,96 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-    </row>
-    <row r="4" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+    </row>
+    <row r="4" spans="1:13" ht="175.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8">
         <v>1</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="12" t="s">
+      <c r="F4" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="12" t="s">
+      <c r="G4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="H4" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="13" t="s">
+      <c r="H4" s="9"/>
+      <c r="I4" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11">
+    <row r="5" spans="1:13" ht="196.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="8">
         <v>2</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="12" t="s">
+      <c r="G5" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="13" t="s">
+      <c r="H5" s="9"/>
+      <c r="I5" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="11">
+    <row r="6" spans="1:13" ht="168" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8">
         <v>3</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="12" t="s">
+      <c r="E6" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="12" t="s">
+      <c r="F6" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="12" t="s">
+      <c r="G6" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="I6" s="13" t="s">
+      <c r="H6" s="9"/>
+      <c r="I6" s="10" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1072,101 +1824,95 @@
       <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8"/>
-    </row>
-    <row r="12" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="11">
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+    </row>
+    <row r="12" spans="1:13" ht="168" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8">
         <v>4</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="E12" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="12" t="s">
+      <c r="F12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="G12" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H12" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="I12" s="13" t="s">
+      <c r="H12" s="9"/>
+      <c r="I12" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="11">
+    <row r="13" spans="1:13" ht="175.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="8">
         <v>5</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="G13" s="12" t="s">
+      <c r="G13" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H13" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="I13" s="13" t="s">
+      <c r="H13" s="9"/>
+      <c r="I13" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="11">
+    <row r="14" spans="1:13" ht="168" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8">
         <v>6</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="12" t="s">
+      <c r="E14" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="H14" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="I14" s="13" t="s">
+      <c r="H14" s="9"/>
+      <c r="I14" s="10" t="s">
         <v>0</v>
       </c>
     </row>
@@ -1191,144 +1937,136 @@
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-    </row>
-    <row r="18" spans="1:9" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="11">
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+    </row>
+    <row r="18" spans="1:9" ht="196.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8">
         <v>7</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="E18" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="12" t="s">
+      <c r="F18" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="12" t="s">
+      <c r="G18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H18" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="I18" s="13" t="s">
+      <c r="H18" s="9"/>
+      <c r="I18" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
+    <row r="19" spans="1:9" ht="168" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="8">
         <v>8</v>
       </c>
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D19" s="12" t="s">
+      <c r="D19" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="12" t="s">
+      <c r="E19" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="12" t="s">
+      <c r="F19" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="G19" s="12" t="s">
+      <c r="G19" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="H19" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="I19" s="14" t="s">
+      <c r="H19" s="9"/>
+      <c r="I19" s="11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="11">
+    <row r="20" spans="1:9" ht="183" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="8">
         <v>9</v>
       </c>
-      <c r="B20" s="12" t="s">
+      <c r="B20" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="D20" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="12" t="s">
+      <c r="E20" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F20" s="12" t="s">
+      <c r="F20" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="G20" s="12" t="s">
+      <c r="G20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="H20" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="I20" s="13" t="s">
+      <c r="H20" s="9"/>
+      <c r="I20" s="10" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="100.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="11">
+    <row r="21" spans="1:9" ht="184.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="8">
         <v>10</v>
       </c>
-      <c r="B21" s="12" t="s">
+      <c r="B21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="D21" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="G21" s="12" t="s">
+      <c r="G21" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="H21" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="I21" s="14" t="s">
+      <c r="H21" s="9"/>
+      <c r="I21" s="11" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1449,5 +2187,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="1200" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Completa casos manuales CP-MAN-11 a CP-MAN-20
</commit_message>
<xml_diff>
--- a/reportes/ejecucion-manual/Plantilla - Casos de prueba - ejecutada.xlsx
+++ b/reportes/ejecucion-manual/Plantilla - Casos de prueba - ejecutada.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/24c0bad5dbd80ad4/Desktop/Proyecto-Aseguramiento y Calidad de software/048-proyecto-final/reportes/ejecucion-manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{4EF7628D-2600-4160-9ACF-98E5AD117BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4DBCA349-3370-498A-9647-9D765A34E176}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{4EF7628D-2600-4160-9ACF-98E5AD117BA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3151CC36-3946-44E4-99BA-85EAEFAB7D5C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detalle de resultados" sheetId="4" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="182">
   <si>
     <t>OK</t>
   </si>
@@ -65,9 +65,6 @@
   </si>
   <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AREA FUNCIONAL : </t>
   </si>
   <si>
     <t>SUITE DE PRUEBAS - OPENCART DEMO</t>
@@ -349,6 +346,277 @@
   </si>
   <si>
     <t>CP-MAN-10-agregado.png; CP-MAN-10-repeticion.png; CP-MAN-10.png</t>
+  </si>
+  <si>
+    <t>AREA FUNCIONAL: CATEGORIAS, CARRITO, CUENTA Y CONTACTO</t>
+  </si>
+  <si>
+    <t>Navegación por categorías</t>
+  </si>
+  <si>
+    <t>Acceso al sitio; página principal</t>
+  </si>
+  <si>
+    <t>Categoría Desktops</t>
+  </si>
+  <si>
+    <t>1. Abrir la página principal.
+2. Seleccionar Desktops y Show All Desktops.
+3. Revisar contenido.</t>
+  </si>
+  <si>
+    <t>Se abre la categoría seleccionada y se muestra el contenido disponible.</t>
+  </si>
+  <si>
+    <t>Se abrió Desktops. La página mostró el encabezado de la categoría, el texto de descripción, categorías refinadas (PC 0, Mac 1) y el listado de productos (13 en el menú).</t>
+  </si>
+  <si>
+    <t>CP-MAN-11</t>
+  </si>
+  <si>
+    <t>CP-MAN-11.png</t>
+  </si>
+  <si>
+    <t>Filtrado y ordenamiento de productos</t>
+  </si>
+  <si>
+    <t>Categoría con varios productos y opciones de ordenamiento</t>
+  </si>
+  <si>
+    <t>Price (Low &gt; High)</t>
+  </si>
+  <si>
+    <t>1. Abrir Desktops.
+2. Seleccionar Price (Low &gt; High).
+3. Revisar nombre y precio de los productos.</t>
+  </si>
+  <si>
+    <t>Los productos aparecen ordenados por precio ascendente.</t>
+  </si>
+  <si>
+    <t>La URL incluyó sort=p.price&amp;order=ASC. Se observaron precios en orden ascendente: $98.00, $110.00, $122.00, $122.00, $122.00, $122.00, $123.20, $242.00, $337.99, $602.00 y valores mayores.</t>
+  </si>
+  <si>
+    <t>CP-MAN-12</t>
+  </si>
+  <si>
+    <t>CP-MAN-12.png</t>
+  </si>
+  <si>
+    <t>Selección de cantidad de un producto</t>
+  </si>
+  <si>
+    <t>Producto con campo de cantidad</t>
+  </si>
+  <si>
+    <t>iPhone; cantidad 2</t>
+  </si>
+  <si>
+    <t>1. Abrir los detalles de iPhone.
+2. Introducir 2 en Qty.
+3. Agregar al carrito.
+4. Revisar cantidad y subtotal.</t>
+  </si>
+  <si>
+    <t>El carrito refleja 2 unidades y calcula el importe correspondiente si la cantidad es válida.</t>
+  </si>
+  <si>
+    <t>Se agregaron 2 unidades; el encabezado mostró 2 items / $246.40 y la línea mostró cantidad 2, precio unitario $123.20 y total $246.40. No obstante, apareció *** y el aviso de falta de stock aunque la ficha indicaba In Stock; reproduce BUG-002.</t>
+  </si>
+  <si>
+    <t>CP-MAN-13</t>
+  </si>
+  <si>
+    <t>CP-MAN-13.png</t>
+  </si>
+  <si>
+    <t>Actualización de cantidad en el carrito</t>
+  </si>
+  <si>
+    <t>Producto con cantidad 1 en carrito</t>
+  </si>
+  <si>
+    <t>Cambiar de 1 a 2 unidades</t>
+  </si>
+  <si>
+    <t>1. Abrir el carrito con una unidad.
+2. Cambiar cantidad a 2.
+3. Pulsar actualizar.
+4. Revisar cantidad y totales; repetir para confirmar una respuesta inesperada.</t>
+  </si>
+  <si>
+    <t>El sistema conserva 2 unidades y recalcula subtotal y totales, o informa claramente si la cantidad no es válida.</t>
+  </si>
+  <si>
+    <t>Primer intento: después de pulsar actualizar, el carrito apareció vacío. En la repetición, la actualización fue confirmada y el carrito conservó 2 iPhone con línea total $246.40 y total general $246.40; se mostró el aviso de falta de stock (***) ya registrado en BUG-002. La anomalía del primer intento no se reprodujo; no se confirma un defecto independiente.</t>
+  </si>
+  <si>
+    <t>OBSERVACIÓN</t>
+  </si>
+  <si>
+    <t>CP-MAN-14</t>
+  </si>
+  <si>
+    <t>CP-MAN-14.png; CP-MAN-14-repeticion.png</t>
+  </si>
+  <si>
+    <t>Eliminación de un producto del carrito</t>
+  </si>
+  <si>
+    <t>iPhone agregado al carrito</t>
+  </si>
+  <si>
+    <t>Producto iPhone en carrito</t>
+  </si>
+  <si>
+    <t>1. Abrir el carrito.
+2. Seleccionar el botón de eliminar del producto.
+3. Revisar contenido y total final.</t>
+  </si>
+  <si>
+    <t>El producto desaparece y el carrito muestra estado vacío o totales actualizados.</t>
+  </si>
+  <si>
+    <t>Se eliminó iPhone; el carrito mostró “Your shopping cart is empty!” y el encabezado pasó a 0 items - $0.00.</t>
+  </si>
+  <si>
+    <t>CP-MAN-15</t>
+  </si>
+  <si>
+    <t>CP-MAN-15.png</t>
+  </si>
+  <si>
+    <t>Agregar producto a lista de deseos</t>
+  </si>
+  <si>
+    <t>Producto visible en catálogo; sesión cerrada</t>
+  </si>
+  <si>
+    <t>iPhone</t>
+  </si>
+  <si>
+    <t>1. Abrir la búsqueda de iPhone.
+2. Pulsar el icono de corazón.
+3. Revisar el mensaje.</t>
+  </si>
+  <si>
+    <t>Se agrega el producto o se informa claramente que se requiere iniciar sesión.</t>
+  </si>
+  <si>
+    <t>Al pulsar el corazón apareció: “You must login or create an account to save iPhone to your wish list!”. No se guardó el producto por estar la sesión cerrada.</t>
+  </si>
+  <si>
+    <t>CP-MAN-16</t>
+  </si>
+  <si>
+    <t>CP-MAN-16.png</t>
+  </si>
+  <si>
+    <t>Validación de correo duplicado en registro</t>
+  </si>
+  <si>
+    <t>Cuenta de prueba existente</t>
+  </si>
+  <si>
+    <t>Correo ya registrado qa.manual.048.20261023.1416@example.com y demás datos ficticios</t>
+  </si>
+  <si>
+    <t>1. Abrir Register.
+2. Completar campos con datos ficticios y el correo ya existente.
+3. Aceptar la política.
+4. Enviar y revisar el mensaje.</t>
+  </si>
+  <si>
+    <t>El sitio rechaza el correo duplicado con un mensaje claro y no crea otra cuenta.</t>
+  </si>
+  <si>
+    <t>El registro fue rechazado y mostró “Warning: E-Mail Address is already registered!”. No se creó otra cuenta; comportamiento esperado.</t>
+  </si>
+  <si>
+    <t>CP-MAN-17</t>
+  </si>
+  <si>
+    <t>CP-MAN-17.png</t>
+  </si>
+  <si>
+    <t>Recuperación de contraseña</t>
+  </si>
+  <si>
+    <t>Formulario de inicio de sesión disponible</t>
+  </si>
+  <si>
+    <t>Correo de una cuenta de prueba existente</t>
+  </si>
+  <si>
+    <t>1. Abrir Login y Forgotten Password.
+2. Introducir el correo de prueba.
+3. Enviar solicitud.
+4. Revisar confirmación; no asumir recepción del correo.</t>
+  </si>
+  <si>
+    <t>El sitio permite solicitar recuperación o informa que la función no está disponible; no se presume entrega del correo.</t>
+  </si>
+  <si>
+    <t>El sitio mostró “An email with a confirmation link has been sent your email address.” La bandeja del correo no fue verificada; solo se confirma el mensaje mostrado en pantalla.</t>
+  </si>
+  <si>
+    <t>CP-MAN-18</t>
+  </si>
+  <si>
+    <t>CP-MAN-18.png</t>
+  </si>
+  <si>
+    <t>Acceso a información de contacto</t>
+  </si>
+  <si>
+    <t>Página principal accesible</t>
+  </si>
+  <si>
+    <t>Opción Contact Us del encabezado</t>
+  </si>
+  <si>
+    <t>1. Abrir la página principal.
+2. Seleccionar Contact Us.
+3. Revisar información y campos visibles.</t>
+  </si>
+  <si>
+    <t>La página de contacto carga y presenta su información y campos principales.</t>
+  </si>
+  <si>
+    <t>La página Contact Us cargó, mostró Your Store, Address 1, teléfono 123456789 y campos Your Name, E-Mail Address y Enquiry.</t>
+  </si>
+  <si>
+    <t>CP-MAN-19</t>
+  </si>
+  <si>
+    <t>CP-MAN-19.png</t>
+  </si>
+  <si>
+    <t>Validación del formulario de contacto</t>
+  </si>
+  <si>
+    <t>Formulario de contacto disponible</t>
+  </si>
+  <si>
+    <t>Formulario vacío</t>
+  </si>
+  <si>
+    <t>1. Abrir Contact Us.
+2. Dejar vacíos los campos.
+3. Pulsar Submit.
+4. Revisar mensajes.</t>
+  </si>
+  <si>
+    <t>El sistema impide el envío incompleto e identifica los campos que requieren atención.</t>
+  </si>
+  <si>
+    <t>El formulario no se envió y mostró validaciones: Name must be between 3 and 32 characters!, E-Mail Address does not appear to be valid! y Enquiry must be between 10 and 3000 characters!.</t>
+  </si>
+  <si>
+    <t>CP-MAN-20</t>
+  </si>
+  <si>
+    <t>CP-MAN-20.png</t>
   </si>
 </sst>
 </file>
@@ -387,7 +655,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -424,6 +692,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -437,7 +711,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -472,6 +746,15 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -484,14 +767,137 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="44">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF9999"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1181,6 +1587,556 @@
         <a:xfrm>
           <a:off x="9199880" y="22611080"/>
           <a:ext cx="1846580" cy="2215046"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>63501</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>1177136</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Imagen 3" descr="CP-MAN-11 - CP-MAN-11.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0143AAD5-40EB-4AE8-9B6D-73DF54E9988F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="25689561"/>
+          <a:ext cx="1846580" cy="1113635"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>63501</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>1177136</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Imagen 11" descr="CP-MAN-12 - CP-MAN-12.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6612AA45-A529-4476-BAB2-0A9EBF39BB50}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="26969721"/>
+          <a:ext cx="1846580" cy="1113635"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>63499</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>2653528</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="Imagen 19" descr="CP-MAN-13 - CP-MAN-13.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{732D6D66-D193-47BF-A9CD-383CDCE3961B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId12" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="28249879"/>
+          <a:ext cx="1846580" cy="2590029"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>2076174</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="24" name="Imagen 23" descr="CP-MAN-14 - CP-MAN-14.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE42E467-194E-4312-810C-F68CB07175E1}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId13" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="31000700"/>
+          <a:ext cx="1587500" cy="2012674"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>2177774</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1651000</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>4502426</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="26" name="Imagen 25" descr="CP-MAN-14 - CP-MAN-14-repeticion.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27DFC64B-24E9-4F11-B981-B1B3628B3113}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="33114974"/>
+          <a:ext cx="1587500" cy="2324652"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>2404642</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Imagen 27" descr="CP-MAN-15 - CP-MAN-15.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0B32091A-EE6B-4E5F-A745-4799ED62A826}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="35610800"/>
+          <a:ext cx="1846580" cy="2341142"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>3067805</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="Imagen 29" descr="CP-MAN-16 - CP-MAN-16.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AEC7608-E9B6-42D5-A678-E86F577A6DAD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="38125400"/>
+          <a:ext cx="1846580" cy="3004305"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>63502</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>2709731</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="32" name="Imagen 31" descr="CP-MAN-17 - CP-MAN-17.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CA94D8C-517D-45C3-A2DF-9A5C6664B072}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="41295322"/>
+          <a:ext cx="1846580" cy="2646229"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>63501</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>2518650</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="34" name="Imagen 33" descr="CP-MAN-18 - CP-MAN-18.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB297375-E4A5-4159-91BA-C62426C42179}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="44114721"/>
+          <a:ext cx="1846580" cy="2455149"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>63501</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>2441575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="36" name="Imagen 35" descr="CP-MAN-19 - CP-MAN-19.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B695EDD4-D947-46B7-AB57-94812945BA3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="46743621"/>
+          <a:ext cx="1846580" cy="2378074"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>63500</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>63502</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1910080</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>2562005</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="38" name="Imagen 37" descr="CP-MAN-20 - CP-MAN-20.png">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35CF8F79-C81D-46A4-BD65-E99B41A5B7B4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9199880" y="49296322"/>
+          <a:ext cx="1846580" cy="2498503"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1455,7 +2411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1F9ADDF-D33F-4C42-B5A1-5813E3A0ACA6}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.77734375" customWidth="1"/>
@@ -1465,157 +2421,297 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="16" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="16" t="s">
+      <c r="D1" s="13" t="s">
         <v>79</v>
-      </c>
-      <c r="D1" s="16" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="7" t="s">
         <v>81</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>87</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>89</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>93</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="7" t="s">
         <v>97</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>100</v>
+    </row>
+    <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A15" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A19" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>166</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A21" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -1626,7 +2722,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M25"/>
+  <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6" style="4" customWidth="1"/>
@@ -1642,17 +2738,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
+      <c r="A1" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="E1" s="16"/>
+      <c r="F1" s="16"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1690,39 +2786,39 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
     </row>
     <row r="4" spans="1:13" ht="175.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D4" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="9" t="s">
+      <c r="G4" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>21</v>
       </c>
       <c r="H4" s="9"/>
       <c r="I4" s="10" t="s">
@@ -1734,22 +2830,22 @@
         <v>2</v>
       </c>
       <c r="B5" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E5" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F5" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="G5" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>28</v>
       </c>
       <c r="H5" s="9"/>
       <c r="I5" s="10" t="s">
@@ -1761,22 +2857,22 @@
         <v>3</v>
       </c>
       <c r="B6" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C6" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="9" t="s">
         <v>33</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>34</v>
       </c>
       <c r="H6" s="9"/>
       <c r="I6" s="10" t="s">
@@ -1824,38 +2920,38 @@
       <c r="H10" s="5"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
+      <c r="A11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="16"/>
+      <c r="F11" s="16"/>
+      <c r="G11" s="16"/>
+      <c r="H11" s="16"/>
     </row>
     <row r="12" spans="1:13" ht="168" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>4</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="E12" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="F12" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="G12" s="9" t="s">
         <v>39</v>
-      </c>
-      <c r="G12" s="9" t="s">
-        <v>40</v>
       </c>
       <c r="H12" s="9"/>
       <c r="I12" s="10" t="s">
@@ -1867,22 +2963,22 @@
         <v>5</v>
       </c>
       <c r="B13" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="E13" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="F13" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="G13" s="9" t="s">
         <v>45</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>46</v>
       </c>
       <c r="H13" s="9"/>
       <c r="I13" s="10" t="s">
@@ -1894,22 +2990,22 @@
         <v>6</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="9" t="s">
+      <c r="F14" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F14" s="9" t="s">
+      <c r="G14" s="9" t="s">
         <v>51</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>52</v>
       </c>
       <c r="H14" s="9"/>
       <c r="I14" s="10" t="s">
@@ -1937,38 +3033,38 @@
       <c r="H16" s="5"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
+      <c r="A17" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
     </row>
     <row r="18" spans="1:9" ht="196.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="8">
         <v>7</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D18" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F18" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="9" t="s">
+      <c r="G18" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>58</v>
       </c>
       <c r="H18" s="9"/>
       <c r="I18" s="10" t="s">
@@ -1980,26 +3076,26 @@
         <v>8</v>
       </c>
       <c r="B19" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="D19" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="D19" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E19" s="9" t="s">
+      <c r="F19" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F19" s="9" t="s">
+      <c r="G19" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>64</v>
       </c>
       <c r="H19" s="9"/>
       <c r="I19" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="183" customHeight="1" x14ac:dyDescent="0.3">
@@ -2007,22 +3103,22 @@
         <v>9</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>12</v>
       </c>
       <c r="D20" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F20" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F20" s="9" t="s">
+      <c r="G20" s="9" t="s">
         <v>69</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>70</v>
       </c>
       <c r="H20" s="9"/>
       <c r="I20" s="10" t="s">
@@ -2034,39 +3130,309 @@
         <v>10</v>
       </c>
       <c r="B21" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="D21" s="9" t="s">
+      <c r="E21" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="F21" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F21" s="9" t="s">
+      <c r="G21" s="9" t="s">
         <v>75</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>76</v>
       </c>
       <c r="H21" s="9"/>
       <c r="I21" s="11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="B25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="16"/>
+      <c r="G25" s="16"/>
+      <c r="H25" s="16"/>
+    </row>
+    <row r="26" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8">
+        <v>11</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C26" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G26" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="H26" s="9"/>
+      <c r="I26" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="100.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="8">
+        <v>12</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C27" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E27" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F27" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="G27" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="H27" s="9"/>
+      <c r="I27" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="217.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="8">
         <v>13</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
+      <c r="B28" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="C28" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="F28" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="G28" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="H28" s="9"/>
+      <c r="I28" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="363" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="8">
+        <v>14</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="G29" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="9"/>
+      <c r="I29" s="14" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="198" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="8">
+        <v>15</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="G30" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="H30" s="9"/>
+      <c r="I30" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="250.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="8">
+        <v>16</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="G31" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="H31" s="9"/>
+      <c r="I31" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="222" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="8">
+        <v>17</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="G32" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="H32" s="9"/>
+      <c r="I32" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="207" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="8">
+        <v>18</v>
+      </c>
+      <c r="B33" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="F33" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="H33" s="9"/>
+      <c r="I33" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="201" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="8">
+        <v>19</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="C34" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="9"/>
+      <c r="I34" s="11" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="210" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="8">
+        <v>20</v>
+      </c>
+      <c r="B35" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C35" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="F35" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="H35" s="9"/>
+      <c r="I35" s="11" t="s">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2077,6 +3443,78 @@
     <mergeCell ref="A17:H17"/>
   </mergeCells>
   <conditionalFormatting sqref="I4 I7:I10">
+    <cfRule type="cellIs" dxfId="43" priority="45" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="46" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I15">
+    <cfRule type="cellIs" dxfId="41" priority="39" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="40" priority="40" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I22:I24">
+    <cfRule type="cellIs" dxfId="39" priority="43" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="38" priority="44" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5">
+    <cfRule type="cellIs" dxfId="37" priority="37" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="36" priority="38" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6">
+    <cfRule type="cellIs" dxfId="35" priority="35" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="34" priority="36" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I12">
+    <cfRule type="cellIs" dxfId="33" priority="33" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="32" priority="34" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I13">
+    <cfRule type="cellIs" dxfId="31" priority="31" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="32" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I14">
+    <cfRule type="cellIs" dxfId="29" priority="29" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="30" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I18">
+    <cfRule type="cellIs" dxfId="27" priority="27" operator="equal">
+      <formula>"FALLO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="28" operator="equal">
+      <formula>"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I19">
     <cfRule type="cellIs" dxfId="25" priority="25" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2084,31 +3522,31 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I15">
-    <cfRule type="cellIs" dxfId="23" priority="19" operator="equal">
+  <conditionalFormatting sqref="I20">
+    <cfRule type="cellIs" dxfId="23" priority="23" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="24" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I22:I24">
-    <cfRule type="cellIs" dxfId="21" priority="23" operator="equal">
+  <conditionalFormatting sqref="I21">
+    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="24" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="22" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I26">
-    <cfRule type="cellIs" dxfId="19" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="19" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="20" operator="equal">
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5">
+  <conditionalFormatting sqref="I27">
     <cfRule type="cellIs" dxfId="17" priority="17" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2116,7 +3554,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I6">
+  <conditionalFormatting sqref="I28">
     <cfRule type="cellIs" dxfId="15" priority="15" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2124,7 +3562,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I12">
+  <conditionalFormatting sqref="I29">
     <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2132,7 +3570,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I13">
+  <conditionalFormatting sqref="I30">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2140,7 +3578,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I14">
+  <conditionalFormatting sqref="I31">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2148,7 +3586,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I18">
+  <conditionalFormatting sqref="I32">
     <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2156,7 +3594,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I19">
+  <conditionalFormatting sqref="I33">
     <cfRule type="cellIs" dxfId="5" priority="5" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2164,7 +3602,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I20">
+  <conditionalFormatting sqref="I34">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>
@@ -2172,7 +3610,7 @@
       <formula>"OK"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I21">
+  <conditionalFormatting sqref="I35">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"FALLO"</formula>
     </cfRule>

</xml_diff>